<commit_message>
Add dates to SpaceX lock-up milestones
</commit_message>
<xml_diff>
--- a/24-spacex-ipo-quality-model/spacex_ipo_quality_model.xlsx
+++ b/24-spacex-ipo-quality-model/spacex_ipo_quality_model.xlsx
@@ -5940,7 +5940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6006,20 +6006,30 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>milestone_date</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>milestone_with_date</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>release_x_base_ipo_float</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>release_pct_basic_common</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>release_pct_post_class_a</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>release_pct_relevant_pool</t>
         </is>
@@ -6078,16 +6088,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M2" t="n">
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>IPO float (2026-06-11)</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" t="n">
+      <c r="P2" t="n">
         <v>4.248709722567172</v>
       </c>
-      <c r="O2" t="n">
+      <c r="Q2" t="n">
         <v>7.527652199187732</v>
       </c>
-      <c r="P2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -6142,16 +6162,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M3" t="n">
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Over-allotment option (2026-07-11)</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
         <v>0.1499999995499999</v>
       </c>
-      <c r="N3" t="n">
+      <c r="P3" t="n">
         <v>0.6373064564731565</v>
       </c>
-      <c r="O3" t="n">
+      <c r="Q3" t="n">
         <v>1.129147826490716</v>
       </c>
-      <c r="P3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -6206,16 +6236,26 @@
           <t>expected_month</t>
         </is>
       </c>
-      <c r="M4" t="n">
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>TBD - likely Aug 2026</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>First earnings release unlock (TBD - likely Aug 2026)</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
         <v>1.6407000016407</v>
       </c>
-      <c r="N4" t="n">
+      <c r="P4" t="n">
         <v>6.970858048786818</v>
       </c>
-      <c r="O4" t="n">
+      <c r="Q4" t="n">
         <v>12.35061897555793</v>
       </c>
-      <c r="P4" t="n">
+      <c r="R4" t="n">
         <v>20</v>
       </c>
     </row>
@@ -6272,16 +6312,26 @@
           <t>expected_month</t>
         </is>
       </c>
-      <c r="M5" t="n">
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>TBD - likely Aug 2026</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Performance early release (TBD - likely Aug 2026)</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
         <v>0.82044000082044</v>
       </c>
-      <c r="N5" t="n">
+      <c r="P5" t="n">
         <v>3.485811408268823</v>
       </c>
-      <c r="O5" t="n">
+      <c r="Q5" t="n">
         <v>6.17598697647757</v>
       </c>
-      <c r="P5" t="n">
+      <c r="R5" t="n">
         <v>10.00109709270433</v>
       </c>
     </row>
@@ -6338,16 +6388,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M6" t="n">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Day 70 release (2026-08-20)</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
         <v>0.5742000005742</v>
       </c>
-      <c r="N6" t="n">
+      <c r="P6" t="n">
         <v>2.43960912513768</v>
       </c>
-      <c r="O6" t="n">
+      <c r="Q6" t="n">
         <v>4.322377897095973</v>
       </c>
-      <c r="P6" t="n">
+      <c r="R6" t="n">
         <v>6.999451453647833</v>
       </c>
     </row>
@@ -6404,16 +6464,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Day 90 release (2026-09-09)</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
         <v>0.5742000005742</v>
       </c>
-      <c r="N7" t="n">
+      <c r="P7" t="n">
         <v>2.43960912513768</v>
       </c>
-      <c r="O7" t="n">
+      <c r="Q7" t="n">
         <v>4.322377897095973</v>
       </c>
-      <c r="P7" t="n">
+      <c r="R7" t="n">
         <v>6.999451453647833</v>
       </c>
     </row>
@@ -6470,16 +6540,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M8" t="n">
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Affiliate catch-up release (2026-09-10)</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
         <v>0.10638000010638</v>
       </c>
-      <c r="N8" t="n">
+      <c r="P8" t="n">
         <v>0.4519777407386735</v>
       </c>
-      <c r="O8" t="n">
+      <c r="Q8" t="n">
         <v>0.8007916417503825</v>
       </c>
-      <c r="P8" t="n">
+      <c r="R8" t="n">
         <v>1.296763576522216</v>
       </c>
     </row>
@@ -6536,16 +6616,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M9" t="n">
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Day 105 release (2026-09-24)</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
         <v>0.5911200005911199</v>
       </c>
-      <c r="N9" t="n">
+      <c r="P9" t="n">
         <v>2.511497293715404</v>
       </c>
-      <c r="O9" t="n">
+      <c r="Q9" t="n">
         <v>4.449745772433598</v>
       </c>
-      <c r="P9" t="n">
+      <c r="R9" t="n">
         <v>7.205704882062534</v>
       </c>
     </row>
@@ -6602,16 +6692,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Day 120 release (2026-10-09)</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
         <v>0.5911200005911199</v>
       </c>
-      <c r="N10" t="n">
+      <c r="P10" t="n">
         <v>2.511497293715404</v>
       </c>
-      <c r="O10" t="n">
+      <c r="Q10" t="n">
         <v>4.449745772433598</v>
       </c>
-      <c r="P10" t="n">
+      <c r="R10" t="n">
         <v>7.205704882062534</v>
       </c>
     </row>
@@ -6668,16 +6768,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Day 135 release (2026-10-24)</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
         <v>0.5911200005911199</v>
       </c>
-      <c r="N11" t="n">
+      <c r="P11" t="n">
         <v>2.511497293715404</v>
       </c>
-      <c r="O11" t="n">
+      <c r="Q11" t="n">
         <v>4.449745772433598</v>
       </c>
-      <c r="P11" t="n">
+      <c r="R11" t="n">
         <v>7.205704882062534</v>
       </c>
     </row>
@@ -6734,16 +6844,26 @@
           <t>expected_month</t>
         </is>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>TBD - likely Nov 2026</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Q3 2026 earnings release unlock (TBD - likely Nov 2026)</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
         <v>2.34000000234</v>
       </c>
-      <c r="N12" t="n">
+      <c r="P12" t="n">
         <v>9.941980760749166</v>
       </c>
-      <c r="O12" t="n">
+      <c r="Q12" t="n">
         <v>17.614706163714</v>
       </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>28.52441031267142</v>
       </c>
     </row>
@@ -6800,16 +6920,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M13" t="n">
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Day 180 final 180-day release (2026-12-08)</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
         <v>0.5911200005911199</v>
       </c>
-      <c r="N13" t="n">
+      <c r="P13" t="n">
         <v>2.511497293715404</v>
       </c>
-      <c r="O13" t="n">
+      <c r="Q13" t="n">
         <v>4.449745772433598</v>
       </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
         <v>7.205704882062534</v>
       </c>
     </row>
@@ -6866,16 +6996,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M14" t="n">
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Day 180 final 180-day release - no performance release case (2026-12-08)</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
         <v>1.43568000143568</v>
       </c>
-      <c r="N14" t="n">
+      <c r="P14" t="n">
         <v>6.099787580595026</v>
       </c>
-      <c r="O14" t="n">
+      <c r="Q14" t="n">
         <v>10.80729972013714</v>
       </c>
-      <c r="P14" t="n">
+      <c r="R14" t="n">
         <v>17.50082281952825</v>
       </c>
     </row>
@@ -6932,16 +7072,26 @@
           <t>expected_month</t>
         </is>
       </c>
-      <c r="M15" t="n">
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>TBD - likely Mar 2027</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Q4 2026 extended-lock release (TBD - likely Mar 2027)</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
         <v>0.63342000063342</v>
       </c>
-      <c r="N15" t="n">
+      <c r="P15" t="n">
         <v>2.691217715159716</v>
       </c>
-      <c r="O15" t="n">
+      <c r="Q15" t="n">
         <v>4.768165460777658</v>
       </c>
-      <c r="P15" t="n">
+      <c r="R15" t="n">
         <v>5.4984375</v>
       </c>
     </row>
@@ -6998,16 +7148,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M16" t="n">
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2027-03-18</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Day 280 extended release (2027-03-18)</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
         <v>0.3168000003168</v>
       </c>
-      <c r="N16" t="n">
+      <c r="P16" t="n">
         <v>1.345991241455271</v>
       </c>
-      <c r="O16" t="n">
+      <c r="Q16" t="n">
         <v>2.384760219087434</v>
       </c>
-      <c r="P16" t="n">
+      <c r="R16" t="n">
         <v>2.75</v>
       </c>
     </row>
@@ -7064,16 +7224,26 @@
           <t>expected_month</t>
         </is>
       </c>
-      <c r="M17" t="n">
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>TBD - likely May 2027</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Q1 2027 extended-lock release (TBD - likely May 2027)</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
         <v>0.63342000063342</v>
       </c>
-      <c r="N17" t="n">
+      <c r="P17" t="n">
         <v>2.691217715159716</v>
       </c>
-      <c r="O17" t="n">
+      <c r="Q17" t="n">
         <v>4.768165460777658</v>
       </c>
-      <c r="P17" t="n">
+      <c r="R17" t="n">
         <v>5.4984375</v>
       </c>
     </row>
@@ -7130,16 +7300,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M18" t="n">
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2027-05-17</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Day 340 extended release (2027-05-17)</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
         <v>0.3168000003168</v>
       </c>
-      <c r="N18" t="n">
+      <c r="P18" t="n">
         <v>1.345991241455271</v>
       </c>
-      <c r="O18" t="n">
+      <c r="Q18" t="n">
         <v>2.384760219087434</v>
       </c>
-      <c r="P18" t="n">
+      <c r="R18" t="n">
         <v>2.75</v>
       </c>
     </row>
@@ -7196,16 +7376,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M19" t="n">
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2027-06-12</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Day 366 extended release (2027-06-12)</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
         <v>0.63342000063342</v>
       </c>
-      <c r="N19" t="n">
+      <c r="P19" t="n">
         <v>2.691217715159716</v>
       </c>
-      <c r="O19" t="n">
+      <c r="Q19" t="n">
         <v>4.768165460777658</v>
       </c>
-      <c r="P19" t="n">
+      <c r="R19" t="n">
         <v>5.4984375</v>
       </c>
     </row>
@@ -7262,16 +7452,26 @@
           <t>model_calendar_date</t>
         </is>
       </c>
-      <c r="M20" t="n">
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2027-06-12</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Musk lock-up release (2027-06-12)</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
         <v>11.52000001152</v>
       </c>
-      <c r="N20" t="n">
+      <c r="P20" t="n">
         <v>48.94513605291896</v>
       </c>
-      <c r="O20" t="n">
+      <c r="Q20" t="n">
         <v>86.71855342136122</v>
       </c>
-      <c r="P20" t="n">
+      <c r="R20" t="n">
         <v>100</v>
       </c>
     </row>
@@ -7328,16 +7528,26 @@
           <t>expected_month</t>
         </is>
       </c>
-      <c r="M21" t="n">
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>TBD - likely Aug 2027</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Q2 2027 remaining extended release (TBD - likely Aug 2027)</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
         <v>0.63342000063342</v>
       </c>
-      <c r="N21" t="n">
+      <c r="P21" t="n">
         <v>2.691217715159716</v>
       </c>
-      <c r="O21" t="n">
+      <c r="Q21" t="n">
         <v>4.768165460777658</v>
       </c>
-      <c r="P21" t="n">
+      <c r="R21" t="n">
         <v>5.4984375</v>
       </c>
     </row>
@@ -7566,7 +7776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:W12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7670,6 +7880,21 @@
           <t>date_precision</t>
         </is>
       </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>milestone_date</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>milestone</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>milestone_with_date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -7746,6 +7971,21 @@
           <t>model_calendar_date</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>IPO float</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>IPO float (2026-06-11)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -7822,6 +8062,21 @@
           <t>expected_month</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>TBD - likely Aug 2026</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>First earnings release unlock</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>First earnings release unlock (TBD - likely Aug 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -7898,6 +8153,21 @@
           <t>expected_month</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>TBD - likely Aug 2026</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Performance early release</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Performance early release (TBD - likely Aug 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -7974,6 +8244,21 @@
           <t>model_calendar_date</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Day 70 release</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>Day 70 release (2026-08-20)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -8050,6 +8335,21 @@
           <t>model_calendar_date</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Day 90 release</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Day 90 release (2026-09-09)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -8126,6 +8426,21 @@
           <t>model_calendar_date</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Affiliate catch-up release</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Affiliate catch-up release (2026-09-10)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -8202,6 +8517,21 @@
           <t>model_calendar_date</t>
         </is>
       </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Day 105 release</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Day 105 release (2026-09-24)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -8278,6 +8608,21 @@
           <t>model_calendar_date</t>
         </is>
       </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Day 120 release</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Day 120 release (2026-10-09)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -8354,6 +8699,21 @@
           <t>model_calendar_date</t>
         </is>
       </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Day 135 release</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Day 135 release (2026-10-24)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -8430,6 +8790,21 @@
           <t>expected_month</t>
         </is>
       </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>TBD - likely Nov 2026</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>Q3 2026 earnings release unlock</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Q3 2026 earnings release unlock (TBD - likely Nov 2026)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -8504,6 +8879,21 @@
       <c r="T12" t="inlineStr">
         <is>
           <t>model_calendar_date</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>2026-12-08</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Day 180 final release</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Day 180 final release (2026-12-08)</t>
         </is>
       </c>
     </row>

</xml_diff>